<commit_message>
docs: HC-SR04 ASCII 메시지 규격 추가
</commit_message>
<xml_diff>
--- a/docs/설계/STM32-WPF-통신-인터페이스-규격서.xlsx
+++ b/docs/설계/STM32-WPF-통신-인터페이스-규격서.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\stm32-baseboard\docs\설계\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5172638-FB41-44AC-8CA6-16BFA816E41A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC93F6F2-3880-414E-B1F7-C4C2F282052F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="14415" xr2:uid="{14A5CBE1-4160-487D-9821-C17DB7C4730E}"/>
   </bookViews>
@@ -30,10 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="219">
-  <si>
-    <t>항목 내용</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="271">
   <si>
     <t>문서명</t>
   </si>
@@ -98,12 +95,6 @@
     <t>결정 사항</t>
   </si>
   <si>
-    <t>미결 사항</t>
-  </si>
-  <si>
-    <t>항목 V1 규격 상태/근거</t>
-  </si>
-  <si>
     <t>물리 경로</t>
   </si>
   <si>
@@ -227,9 +218,6 @@
     <t>고장</t>
   </si>
   <si>
-    <t>시험 ID 대상 입력/고장 주입 기대 결과 실제 결과 증거 파일 판정</t>
-  </si>
-  <si>
     <t>ICD-T-001</t>
   </si>
   <si>
@@ -278,18 +266,12 @@
     <t>ICD-T-010</t>
   </si>
   <si>
-    <t>개정 날짜 변경 내용 작성 주체 상태</t>
-  </si>
-  <si>
     <t>0.1-draft</t>
   </si>
   <si>
     <t>Codex (사용자 요청)</t>
   </si>
   <si>
-    <t>0.2-draft / 설계 초안 / 사용자 검토 필요</t>
-  </si>
-  <si>
     <t>main.c의 ASCII START/STOP 임시 수신 코드를 단일 라인 수신기와 명령 파서 구조로 정리해야 한다. 본 규격은 아직 구현·시험되지 않았다.</t>
   </si>
   <si>
@@ -302,9 +284,6 @@
     <t>터미널로 직접 송수신을 확인할 수 있고 초기 디버깅이 쉬우며, 현재 ST-LINK Virtual COM Port 환경에서 바이너리 CRC의 복잡도가 필수적이지 않다.</t>
   </si>
   <si>
-    <t>상세 로그 이벤트와 파라미터 조회·설정 명령은 관련 요구사항 승인 후 후속 개정한다.</t>
-  </si>
-  <si>
     <t>문자 집합</t>
   </si>
   <si>
@@ -374,9 +353,6 @@
     <t>START&lt;CR&gt;&lt;LF&gt; = 53 54 41 52 54 0D 0A</t>
   </si>
   <si>
-    <t>구분 형식 필수 여부 설명 검증 규칙 예</t>
-  </si>
-  <si>
     <t>요청</t>
   </si>
   <si>
@@ -503,9 +479,6 @@
     <t>초과 시 CRLF까지 폐기 후 재동기화</t>
   </si>
   <si>
-    <t>방향 명령 요청 라인 정상 응답 오류 응답 예 허용 조건 상태</t>
-  </si>
-  <si>
     <t>PC→MCU / MCU→PC</t>
   </si>
   <si>
@@ -687,13 +660,199 @@
   </si>
   <si>
     <t>사용자 결정·Codex 기록</t>
+  </si>
+  <si>
+    <t>항목</t>
+  </si>
+  <si>
+    <t>내용</t>
+  </si>
+  <si>
+    <t>V1 규격</t>
+  </si>
+  <si>
+    <t>상태/근거</t>
+  </si>
+  <si>
+    <t>구분</t>
+  </si>
+  <si>
+    <t>형식</t>
+  </si>
+  <si>
+    <t>필수 여부</t>
+  </si>
+  <si>
+    <t>설명</t>
+  </si>
+  <si>
+    <t>검증 규칙</t>
+  </si>
+  <si>
+    <t>예</t>
+  </si>
+  <si>
+    <t>방향</t>
+  </si>
+  <si>
+    <t>명령</t>
+  </si>
+  <si>
+    <t>요청 라인</t>
+  </si>
+  <si>
+    <t>정상 응답/발행 라인</t>
+  </si>
+  <si>
+    <t>오류 응답 예</t>
+  </si>
+  <si>
+    <t>허용 조건/발행 조건</t>
+  </si>
+  <si>
+    <t>상태</t>
+  </si>
+  <si>
+    <t>시험 ID</t>
+  </si>
+  <si>
+    <t>대상</t>
+  </si>
+  <si>
+    <t>입력/고장 주입</t>
+  </si>
+  <si>
+    <t>기대 결과</t>
+  </si>
+  <si>
+    <t>실제 결과</t>
+  </si>
+  <si>
+    <t>증거 파일</t>
+  </si>
+  <si>
+    <t>판정</t>
+  </si>
+  <si>
+    <t>개정</t>
+  </si>
+  <si>
+    <t>날짜</t>
+  </si>
+  <si>
+    <t>변경 내용</t>
+  </si>
+  <si>
+    <t>작성 주체</t>
+  </si>
+  <si>
+    <t>0.3-draft / 설계 초안 / 사용자 검토 필요</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>이번 구현 승인</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-09-01 사용자 승인: WPF에서 START·STOP·GET_STATUS 및 HC-SR04 정상·범위 밖·시간초과 데이터 확인</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCU→PC</t>
+  </si>
+  <si>
+    <t>HCSR04_OK</t>
+  </si>
+  <si>
+    <t>발행형 데이터</t>
+  </si>
+  <si>
+    <t>DATA,HCSR04,OK,&lt;DIST_CM&gt;,&lt;PULSE_US&gt;&lt;CR&gt;&lt;LF&gt;</t>
+  </si>
+  <si>
+    <t>해당 없음</t>
+  </si>
+  <si>
+    <t>정상 유효 범위 측정 완료 시</t>
+  </si>
+  <si>
+    <t>HCSR04_OUT_OF_RANGE</t>
+  </si>
+  <si>
+    <t>DATA,HCSR04,OUT_OF_RANGE,0,&lt;PULSE_US&gt;&lt;CR&gt;&lt;LF&gt;</t>
+  </si>
+  <si>
+    <t>Echo 펄스가 설정 유효 범위를 벗어날 때</t>
+  </si>
+  <si>
+    <t>HCSR04_TIMEOUT</t>
+  </si>
+  <si>
+    <t>DATA,HCSR04,TIMEOUT,0,0&lt;CR&gt;&lt;LF&gt;</t>
+  </si>
+  <si>
+    <t>상승 또는 하강 에지 제한시간 초과 시</t>
+  </si>
+  <si>
+    <t>ICD-T-012</t>
+  </si>
+  <si>
+    <t>HC-SR04 정상 데이터</t>
+  </si>
+  <si>
+    <t>DATA,HCSR04,OK,25,1450&lt;CR&gt;&lt;LF&gt;</t>
+  </si>
+  <si>
+    <t>WPF가 상태 OK, 거리 25 cm, 펄스 1450 us로 표시</t>
+  </si>
+  <si>
+    <t>ICD-T-013</t>
+  </si>
+  <si>
+    <t>HC-SR04 범위 밖</t>
+  </si>
+  <si>
+    <t>DATA,HCSR04,OUT_OF_RANGE,0,25000&lt;CR&gt;&lt;LF&gt;</t>
+  </si>
+  <si>
+    <t>WPF가 OUT_OF_RANGE와 펄스폭을 표시</t>
+  </si>
+  <si>
+    <t>ICD-T-014</t>
+  </si>
+  <si>
+    <t>HC-SR04 시간초과</t>
+  </si>
+  <si>
+    <t>WPF가 TIMEOUT을 표시하고 거리값을 유효값으로 취급하지 않음</t>
+  </si>
+  <si>
+    <t>ICD-T-015</t>
+  </si>
+  <si>
+    <t>현재 임시 출력 호환</t>
+  </si>
+  <si>
+    <t>HCSR04 OK DIST_CM=25 PULSE_US=1450&lt;CR&gt;&lt;LF&gt;</t>
+  </si>
+  <si>
+    <t>전환 기간 동안 WPF가 동일 측정값으로 표시</t>
+  </si>
+  <si>
+    <t>0.3-draft</t>
+  </si>
+  <si>
+    <t>사용자 승인 범위에 HC-SR04 정상·범위 밖·시간초과 ASCII 데이터 메시지와 WPF 시험 항목 추가</t>
+  </si>
+  <si>
+    <t>사용자 승인·Codex 기록</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -723,14 +882,6 @@
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
@@ -787,7 +938,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -800,16 +951,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1135,29 +1280,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
+        <v>210</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>85</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2">
         <v>46266</v>
@@ -1165,98 +1312,98 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="27" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="1" t="s">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="27" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="27" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="27" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>22</v>
+        <v>239</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>90</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -1278,174 +1425,178 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C5" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="C6" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="C13" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="B15" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C15" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C11" s="4" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="C16" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1468,191 +1619,201 @@
     <col min="7" max="7" width="37.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="27" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="27" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-    </row>
-    <row r="2" spans="1:6" ht="54" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="E3" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="F3" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D2" s="4" t="s">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="C4" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="54" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="E4" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="F4" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D3" s="4" t="s">
+    </row>
+    <row r="5" spans="1:6" ht="27" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="C5" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="67.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="E5" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="F5" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D4" s="4" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="27" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="C6" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="81" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="E6" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="F6" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D5" s="4" t="s">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="C7" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="E7" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="67.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="F7" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B6" s="4" t="s">
+    </row>
+    <row r="8" spans="1:6" ht="27" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="B8" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="D8" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="E8" s="1" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="B9" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="C9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="E9" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="F9" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C8" s="4" t="s">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="B10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E10" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" spans="1:6" ht="67.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="81" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="F10" s="4"/>
+      <c r="F10" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1662,200 +1823,231 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE2BD567-865E-445A-8672-E2AF96009B63}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.375" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="4.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="7" customFormat="1" ht="81" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="5" customFormat="1" ht="27" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-    </row>
-    <row r="2" spans="1:7" ht="81" x14ac:dyDescent="0.3">
+        <v>220</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="67.5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="54" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="54" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>167</v>
-      </c>
       <c r="G4" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="81" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="54" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>169</v>
+        <v>241</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>49</v>
+        <v>250</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" ht="67.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>172</v>
-      </c>
+        <v>243</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:7" ht="54" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>175</v>
-      </c>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>177</v>
-      </c>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>179</v>
+        <v>46</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>180</v>
+        <v>161</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:7" ht="54" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="67.5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>181</v>
+        <v>162</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>182</v>
+        <v>163</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -1864,68 +2056,82 @@
     </row>
     <row r="13" spans="1:7" ht="54" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>183</v>
+        <v>164</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>185</v>
+        <v>166</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+    <row r="14" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>168</v>
+      </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+    <row r="15" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>171</v>
+      </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+    <row r="16" spans="1:7" ht="54" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>173</v>
+      </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="54" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="1"/>
+        <v>175</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>176</v>
+      </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>55</v>
-      </c>
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1933,12 +2139,8 @@
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>57</v>
-      </c>
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1946,24 +2148,22 @@
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>59</v>
-      </c>
+      <c r="A20" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="27" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>60</v>
+        <v>178</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -1973,10 +2173,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -1986,16 +2186,68 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -2005,7 +2257,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E68C0E0-E0A2-4048-84B2-C4DB5C3ED3D7}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.875" bestFit="1" customWidth="1"/>
@@ -2016,224 +2268,312 @@
     <col min="7" max="7" width="6.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="94.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="27" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C3" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="B4" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="C7" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="D7" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="27" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="C8" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="B11" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="C11" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="27" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="D11" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="B12" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="27" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B9" s="4" t="s">
+      <c r="C12" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="D12" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4" t="s">
-        <v>68</v>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="54" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="54" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="81" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2244,57 +2584,82 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10909A18-DF42-402A-BDBB-6CA6D9DF63D7}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="54" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" ht="81" x14ac:dyDescent="0.3">
+        <v>234</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="67.5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B2" s="2">
         <v>46266</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="94.5" x14ac:dyDescent="0.3">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="81" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2">
         <v>46266</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="121.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>